<commit_message>
feat(drafts): hub phase A — review fixes, JS sources, adapter configs, parity + exec tests (plan 16)
</commit_message>
<xml_diff>
--- a/docs/sheets/mach.xlsx
+++ b/docs/sheets/mach.xlsx
@@ -16,9 +16,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$J$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Commands'!$A$1:$I$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Flags'!$A$1:$E$96</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Functions'!$A$1:$D$453</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Commands'!$A$1:$I$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Flags'!$A$1:$E$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Functions'!$A$1:$D$457</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Config keys'!$A$1:$D$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Destinations'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Templates'!$A$1:$C$8</definedName>
@@ -207,11 +207,11 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-08</t>
+          <t xml:space="preserve">2026-10-15</t>
         </is>
       </c>
       <c r="J2" s="3">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3">
@@ -257,11 +257,11 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-08</t>
+          <t xml:space="preserve">2026-10-15</t>
         </is>
       </c>
       <c r="J3" s="3">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4">
@@ -307,11 +307,11 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-08</t>
+          <t xml:space="preserve">2026-10-15</t>
         </is>
       </c>
       <c r="J4" s="3">
-        <v>452</v>
+        <v>456</v>
       </c>
     </row>
     <row r="5">
@@ -357,7 +357,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-08</t>
+          <t xml:space="preserve">2026-10-15</t>
         </is>
       </c>
       <c r="J5" s="3">
@@ -521,11 +521,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
     <col min="3" max="3" width="60" customWidth="1"/>
     <col min="4" max="4" width="60" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
@@ -1077,22 +1077,27 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">inventory</t>
+          <t xml:space="preserve">inbox</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pull-drafts</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach inventory [--host H] [--section S] [--light|--full] [--diff] [--apply]</t>
+          <t xml:space="preserve">mach inbox pull-drafts [--apply] [--json] [--limit N]</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Regenerate inventory/&lt;host&gt;/ for this machine, show the diff, write only with --apply</t>
+          <t xml:space="preserve">Bring tagged Drafts from the Mac into the synced mach inbox</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">upkeep</t>
+          <t xml:space="preserve">gateway</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1119,22 +1124,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mcp</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">render</t>
+          <t xml:space="preserve">inventory</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach mcp [render] [--tool T]</t>
+          <t xml:space="preserve">mach inventory [--host H] [--section S] [--light|--full] [--diff] [--apply]</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Render (dry-run) or apply the MCP server manifest for each tool via scripts/mcp-apply.sh</t>
+          <t xml:space="preserve">Regenerate inventory/&lt;host&gt;/ for this machine, show the diff, write only with --apply</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1149,12 +1149,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1171,12 +1171,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">apply</t>
+          <t xml:space="preserve">render</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach mcp apply [--tool T] [--apply]</t>
+          <t xml:space="preserve">mach mcp [render] [--tool T]</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1191,17 +1191,17 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">stub</t>
+          <t xml:space="preserve">working</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1213,22 +1213,22 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">memory</t>
+          <t xml:space="preserve">mcp</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">init</t>
+          <t xml:space="preserve">apply</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach memory init [--reindex] [--apply] [--json]</t>
+          <t xml:space="preserve">mach mcp apply [--tool T] [--apply]</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Set up and review lessons (init skeleton, duplicates, stale, caps); collect/promote are preview-only in v1</t>
+          <t xml:space="preserve">Render (dry-run) or apply the MCP server manifest for each tool via scripts/mcp-apply.sh</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">working</t>
+          <t xml:space="preserve">stub</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1265,12 +1265,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">review</t>
+          <t xml:space="preserve">init</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach memory review [--save] [--apply] [--json]</t>
+          <t xml:space="preserve">mach memory init [--reindex] [--apply] [--json]</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1312,17 +1312,17 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">collect</t>
+          <t xml:space="preserve">review</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach memory collect</t>
+          <t xml:space="preserve">mach memory review [--save] [--apply] [--json]</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PREVIEW-ONLY in v1: lists raw memory files it would turn into proposed lessons</t>
+          <t xml:space="preserve">Set up and review lessons (init skeleton, duplicates, stale, caps); collect/promote are preview-only in v1</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1332,17 +1332,17 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">preview-only</t>
+          <t xml:space="preserve">working</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1359,17 +1359,17 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">promote</t>
+          <t xml:space="preserve">collect</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach memory promote</t>
+          <t xml:space="preserve">mach memory collect</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PREVIEW-ONLY in v1: lists promotion candidates for AGENTS.md; changes nothing</t>
+          <t xml:space="preserve">PREVIEW-ONLY in v1: lists raw memory files it would turn into proposed lessons</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1401,17 +1401,22 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">names</t>
+          <t xml:space="preserve">memory</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">promote</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach names [--fix] [--apply]</t>
+          <t xml:space="preserve">mach memory promote</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check that CLI agent names are explicit (cursor-agent, grokcli-agent, no bare `agent`)</t>
+          <t xml:space="preserve">PREVIEW-ONLY in v1: lists promotion candidates for AGENTS.md; changes nothing</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1421,17 +1426,17 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">working</t>
+          <t xml:space="preserve">preview-only</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1443,22 +1448,22 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">note</t>
+          <t xml:space="preserve">names</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach note "text"; mach note agenda|drafts|inbox|&lt;name&gt; "text"; mach note --to agenda -- "text that may start with a destination name" pbpaste | mach note drafts; mach note [dest] "text" [-t TITLE] [--tag X ...] [--tags a,b] [--project P] [--date D] [--flag] [--open] [--file PATH] [--dry-run] [--json]</t>
+          <t xml:space="preserve">mach names [--fix] [--apply]</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quick capture to inbox, Agenda, Drafts or a named destination</t>
+          <t xml:space="preserve">Check that CLI agent names are explicit (cursor-agent, grokcli-agent, no bare `agent`)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">gateway</t>
+          <t xml:space="preserve">upkeep</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1473,12 +1478,12 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">no</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
     </row>
@@ -1488,19 +1493,14 @@
           <t xml:space="preserve">note</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">flush</t>
-        </is>
-      </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach note flush [--apply]</t>
+          <t xml:space="preserve">mach note "text"; mach note agenda|drafts|inbox|&lt;name&gt; "text"; mach note --to agenda -- "text that may start with a destination name" pbpaste | mach note drafts; mach note [dest] "text" [-t TITLE] [--tag X ...] [--tags a,b] [--project P] [--date D] [--flag] [--open] [--file PATH] [--dry-run] [--json]</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">macOS: deliver outbox items to Agenda/Drafts</t>
+          <t xml:space="preserve">Quick capture to inbox, Agenda, Drafts or a named destination</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1520,34 +1520,39 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">onboard</t>
+          <t xml:space="preserve">note</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">flush</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach onboard [--apply] [--skip-previews]</t>
+          <t xml:space="preserve">mach note flush [--apply]</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Checklist for a new machine: prerequisites, link mach, Syncthing pairing, then previews</t>
+          <t xml:space="preserve">macOS: deliver outbox items to Agenda/Drafts</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">upkeep</t>
+          <t xml:space="preserve">gateway</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1574,22 +1579,17 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">plans</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">list</t>
+          <t xml:space="preserve">onboard</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach plans list [--json]</t>
+          <t xml:space="preserve">mach onboard [--apply] [--skip-previews]</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">List plans with open/total checkbox counts; archive a finished plan (plans/README.md section 4)</t>
+          <t xml:space="preserve">Checklist for a new machine: prerequisites, link mach, Syncthing pairing, then previews</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1604,12 +1604,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1626,12 +1626,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">archive</t>
+          <t xml:space="preserve">list</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach plans archive &lt;NN|file&gt; [--apply] [--force]</t>
+          <t xml:space="preserve">mach plans list [--json]</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1651,12 +1651,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1668,22 +1668,27 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">queue</t>
+          <t xml:space="preserve">plans</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">archive</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach queue [--due today|YYYY-MM-DD] [--json]</t>
+          <t xml:space="preserve">mach plans archive &lt;NN|file&gt; [--apply] [--force]</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">List queued runs, runs waiting for approval, inbox prompts not yet run, and outbox items</t>
+          <t xml:space="preserve">List plans with open/total checkbox counts; archive a finished plan (plans/README.md section 4)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">gateway</t>
+          <t xml:space="preserve">upkeep</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1693,12 +1698,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1710,17 +1715,17 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">reject</t>
+          <t xml:space="preserve">queue</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach reject &lt;id&gt; "reason"</t>
+          <t xml:space="preserve">mach queue [--due today|YYYY-MM-DD] [--json]</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reject (cancel) a run that is waiting at a gate or queued</t>
+          <t xml:space="preserve">List queued runs, runs waiting for approval, inbox prompts not yet run, and outbox items</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1735,7 +1740,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1752,17 +1757,17 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">research</t>
+          <t xml:space="preserve">reject</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach research "&lt;question&gt;" [--depth quick|deep] [--tool T] [--dry-run] [--json]</t>
+          <t xml:space="preserve">mach reject &lt;id&gt; "reason"</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Answer a question with sources (quick), or start the research-to-plan flow (deep)</t>
+          <t xml:space="preserve">Reject (cancel) a run that is waiting at a gate or queued</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1787,24 +1792,24 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">run</t>
+          <t xml:space="preserve">research</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach run &lt;file.md&gt; [--dry-run] [--queue] [--json] [--tool T] [--path P] [--machine M] [--write]; mach run --inbox [--dry-run] [--json]</t>
+          <t xml:space="preserve">mach research "&lt;question&gt;" [--depth quick|deep] [--tool T] [--dry-run] [--json]</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Run a prompt document (task, research or flow brief): validate, plan, record, execute</t>
+          <t xml:space="preserve">Answer a question with sources (quick), or start the research-to-plan flow (deep)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1836,27 +1841,22 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">services</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">check</t>
+          <t xml:space="preserve">run</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach services [check]; mach services [check] --update</t>
+          <t xml:space="preserve">mach run &lt;file.md&gt; [--dry-run] [--queue] [--json] [--tool T] [--path P] [--machine M] [--write]; mach run --inbox [--dry-run] [--json]</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">default: compare live units with the index files</t>
+          <t xml:space="preserve">Run a prompt document (task, research or flow brief): validate, plan, record, execute</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">upkeep</t>
+          <t xml:space="preserve">gateway</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1866,17 +1866,17 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">no</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no</t>
-        </is>
-      </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
     </row>
@@ -1888,17 +1888,17 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">show</t>
+          <t xml:space="preserve">check</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach services show</t>
+          <t xml:space="preserve">mach services [check]; mach services [check] --update</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">print the rows parsed from 75 and 76 for this host</t>
+          <t xml:space="preserve">default: compare live units with the index files</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1930,22 +1930,22 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">sheets</t>
+          <t xml:space="preserve">services</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">lint</t>
+          <t xml:space="preserve">show</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach sheets lint &lt;dir&gt; [--json]</t>
+          <t xml:space="preserve">mach services show</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sheet sets: lint, build (CSVs -&gt; xlsx), scaffold and refresh a folder of index.csv + CSV files + a generated workbook</t>
+          <t xml:space="preserve">print the rows parsed from 75 and 76 for this host</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1982,12 +1982,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">build</t>
+          <t xml:space="preserve">lint</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach sheets build &lt;dir&gt; [--dry-run] [--json]</t>
+          <t xml:space="preserve">mach sheets lint &lt;dir&gt; [--json]</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
     </row>
@@ -2029,12 +2029,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">new</t>
+          <t xml:space="preserve">build</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach sheets new &lt;dir&gt; [--apply]</t>
+          <t xml:space="preserve">mach sheets build &lt;dir&gt; [--dry-run] [--json]</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2059,12 +2059,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no</t>
         </is>
       </c>
     </row>
@@ -2076,12 +2076,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">refresh</t>
+          <t xml:space="preserve">new</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach sheets refresh &lt;set&gt; [--build] [--check] [--dry-run] [--out DIR]</t>
+          <t xml:space="preserve">mach sheets new &lt;dir&gt; [--apply]</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2106,34 +2106,39 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">no</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">sheets</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">refresh</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach status [id] [--status S] [-n N] [--all] [--json]</t>
+          <t xml:space="preserve">mach sheets refresh &lt;set&gt; [--build] [--check] [--dry-run] [--out DIR]</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Show recent runs and their state, or one run in detail</t>
+          <t xml:space="preserve">Sheet sets: lint, build (CSVs -&gt; xlsx), scaffold and refresh a folder of index.csv + CSV files + a generated workbook</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">gateway</t>
+          <t xml:space="preserve">upkeep</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2143,39 +2148,34 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">no</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no</t>
-        </is>
-      </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">subsystem</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">list</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach subsystem list</t>
+          <t xml:space="preserve">mach status [id] [--status S] [-n N] [--all] [--json]</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manage subsystem manifests and send prompts to unit roles</t>
+          <t xml:space="preserve">Show recent runs and their state, or one run in detail</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2212,12 +2212,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">show</t>
+          <t xml:space="preserve">list</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach subsystem show &lt;id&gt;</t>
+          <t xml:space="preserve">mach subsystem list</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2259,12 +2259,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">lint</t>
+          <t xml:space="preserve">show</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach subsystem lint [id]</t>
+          <t xml:space="preserve">mach subsystem show &lt;id&gt;</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2306,12 +2306,12 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">new</t>
+          <t xml:space="preserve">lint</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach subsystem new &lt;id&gt; [--from D] [--apply] [--replace]</t>
+          <t xml:space="preserve">mach subsystem lint [id]</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2331,12 +2331,12 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2353,12 +2353,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">unit</t>
+          <t xml:space="preserve">new</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach subsystem unit &lt;id&gt; --from D [--apply]</t>
+          <t xml:space="preserve">mach subsystem new &lt;id&gt; [--from D] [--apply] [--replace]</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2400,12 +2400,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">role</t>
+          <t xml:space="preserve">unit</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mach subsystem role &lt;id&gt; --from D [--apply]</t>
+          <t xml:space="preserve">mach subsystem unit &lt;id&gt; --from D [--apply]</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2442,53 +2442,100 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">subsystem</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">role</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mach subsystem role &lt;id&gt; --from D [--apply]</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manage subsystem manifests and send prompts to unit roles</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gateway</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">working</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">&lt;subsystem&gt;</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">mach &lt;subsystem&gt; [unit] [prompt] [--role R|--to D] [--roles] [--reply chat|inbox] [--write] [--force] [--dry-run] [--json]</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Manage subsystem manifests and send prompts to unit roles</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">subsystem</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">working</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">no</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I43"/>
+  <autoFilter ref="A1:I44"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -3285,76 +3332,66 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">inventory</t>
+          <t xml:space="preserve">inbox</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--host</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">H</t>
+          <t xml:space="preserve">--apply</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Act on this host</t>
+          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">this machine</t>
+          <t xml:space="preserve">preview</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">inventory</t>
+          <t xml:space="preserve">inbox</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--section</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">S</t>
+          <t xml:space="preserve">--json</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">regenerate only this section</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">all sections</t>
+          <t xml:space="preserve">Machine-readable JSON output</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">inventory</t>
+          <t xml:space="preserve">inbox</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--light</t>
+          <t xml:space="preserve">--limit</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">skip the slow size, network and brew checks</t>
+          <t xml:space="preserve">maximum number of tagged drafts to inspect in one run</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">on for macOS</t>
+          <t xml:space="preserve">50</t>
         </is>
       </c>
     </row>
@@ -3366,17 +3403,22 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--full</t>
+          <t xml:space="preserve">--host</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">run the full generator</t>
+          <t xml:space="preserve">Act on this host</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">on for Linux</t>
+          <t xml:space="preserve">this machine</t>
         </is>
       </c>
     </row>
@@ -3388,17 +3430,22 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--diff</t>
+          <t xml:space="preserve">--section</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">show the diff only</t>
+          <t xml:space="preserve">regenerate only this section</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">off</t>
+          <t xml:space="preserve">all sections</t>
         </is>
       </c>
     </row>
@@ -3410,127 +3457,132 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--apply</t>
+          <t xml:space="preserve">--light</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
+          <t xml:space="preserve">skip the slow size, network and brew checks</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">preview</t>
+          <t xml:space="preserve">on for macOS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mcp</t>
+          <t xml:space="preserve">inventory</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--tool</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T</t>
+          <t xml:space="preserve">--full</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AI tool to use</t>
+          <t xml:space="preserve">run the full generator</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">routes.default_tool (claude)</t>
+          <t xml:space="preserve">on for Linux</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mcp</t>
+          <t xml:space="preserve">inventory</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--apply</t>
+          <t xml:space="preserve">--diff</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
+          <t xml:space="preserve">show the diff only</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">preview</t>
+          <t xml:space="preserve">off</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">memory</t>
+          <t xml:space="preserve">inventory</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--reindex</t>
+          <t xml:space="preserve">--apply</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">regenerate INDEX.md (only when it carries the mach marker)</t>
+          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">off</t>
+          <t xml:space="preserve">preview</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">memory</t>
+          <t xml:space="preserve">mcp</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--apply</t>
+          <t xml:space="preserve">--tool</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
+          <t xml:space="preserve">AI tool to use</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">preview</t>
+          <t xml:space="preserve">routes.default_tool (claude)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">memory</t>
+          <t xml:space="preserve">mcp</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--json</t>
+          <t xml:space="preserve">--apply</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine-readable JSON output</t>
+          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">preview</t>
         </is>
       </c>
     </row>
@@ -3542,12 +3594,12 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--save</t>
+          <t xml:space="preserve">--reindex</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">write the review to the reviews folder as YYYY-MM.md</t>
+          <t xml:space="preserve">regenerate INDEX.md (only when it carries the mach marker)</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -3559,120 +3611,105 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">names</t>
+          <t xml:space="preserve">memory</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--fix</t>
+          <t xml:space="preserve">--apply</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">repair names that are not explicit</t>
+          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">off (check only)</t>
+          <t xml:space="preserve">preview</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">names</t>
+          <t xml:space="preserve">memory</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--apply</t>
+          <t xml:space="preserve">--json</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">preview</t>
+          <t xml:space="preserve">Machine-readable JSON output</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">note</t>
+          <t xml:space="preserve">memory</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--to</t>
+          <t xml:space="preserve">--save</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">destination (use when the text may start with a destination name)</t>
+          <t xml:space="preserve">write the review to the reviews folder as YYYY-MM.md</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">note.default</t>
+          <t xml:space="preserve">off</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">note</t>
+          <t xml:space="preserve">names</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">-t</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TITLE</t>
+          <t xml:space="preserve">--fix</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">note title</t>
+          <t xml:space="preserve">repair names that are not explicit</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">first words of the text</t>
+          <t xml:space="preserve">off (check only)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">note</t>
+          <t xml:space="preserve">names</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--tag</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
+          <t xml:space="preserve">--apply</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tag to add (repeatable)</t>
+          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">none</t>
+          <t xml:space="preserve">preview</t>
         </is>
       </c>
     </row>
@@ -3684,17 +3721,17 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--tags</t>
+          <t xml:space="preserve">--to</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">comma-separated tags</t>
+          <t xml:space="preserve">destination (use when the text may start with a destination name)</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">none</t>
+          <t xml:space="preserve">note.default</t>
         </is>
       </c>
     </row>
@@ -3706,22 +3743,22 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--project</t>
+          <t xml:space="preserve">-t</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P</t>
+          <t xml:space="preserve">TITLE</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Agenda project</t>
+          <t xml:space="preserve">note title</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">note.agenda.project (Inbox)</t>
+          <t xml:space="preserve">first words of the text</t>
         </is>
       </c>
     </row>
@@ -3733,17 +3770,17 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--date</t>
+          <t xml:space="preserve">--tag</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">D</t>
+          <t xml:space="preserve">X</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">date for the note, YYYY-MM-DD</t>
+          <t xml:space="preserve">tag to add (repeatable)</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -3760,17 +3797,17 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--flag</t>
+          <t xml:space="preserve">--tags</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">flag the note in the target app</t>
+          <t xml:space="preserve">comma-separated tags</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">off</t>
+          <t xml:space="preserve">none</t>
         </is>
       </c>
     </row>
@@ -3782,17 +3819,22 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--open</t>
+          <t xml:space="preserve">--project</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">open the note in its app after capture</t>
+          <t xml:space="preserve">Agenda project</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">off</t>
+          <t xml:space="preserve">note.agenda.project (Inbox)</t>
         </is>
       </c>
     </row>
@@ -3804,22 +3846,22 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--file</t>
+          <t xml:space="preserve">--date</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PATH</t>
+          <t xml:space="preserve">D</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">read the note text from this file</t>
+          <t xml:space="preserve">date for the note, YYYY-MM-DD</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">stdin or the text argument</t>
+          <t xml:space="preserve">none</t>
         </is>
       </c>
     </row>
@@ -3831,12 +3873,17 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--dry-run</t>
+          <t xml:space="preserve">--flag</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Show what would happen and change nothing</t>
+          <t xml:space="preserve">flag the note in the target app</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">off</t>
         </is>
       </c>
     </row>
@@ -3848,12 +3895,17 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--json</t>
+          <t xml:space="preserve">--open</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine-readable JSON output</t>
+          <t xml:space="preserve">open the note in its app after capture</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">off</t>
         </is>
       </c>
     </row>
@@ -3865,85 +3917,85 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--apply</t>
+          <t xml:space="preserve">--file</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PATH</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
+          <t xml:space="preserve">read the note text from this file</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">preview</t>
+          <t xml:space="preserve">stdin or the text argument</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">onboard</t>
+          <t xml:space="preserve">note</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--apply</t>
+          <t xml:space="preserve">--dry-run</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">preview</t>
+          <t xml:space="preserve">Show what would happen and change nothing</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">onboard</t>
+          <t xml:space="preserve">note</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--skip-previews</t>
+          <t xml:space="preserve">--json</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">skip the inventory, names, ai and mcp previews</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">off</t>
+          <t xml:space="preserve">Machine-readable JSON output</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">plans</t>
+          <t xml:space="preserve">note</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--json</t>
+          <t xml:space="preserve">--apply</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine-readable JSON output</t>
+          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">preview</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">plans</t>
+          <t xml:space="preserve">onboard</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -3965,132 +4017,122 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">plans</t>
+          <t xml:space="preserve">onboard</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--force</t>
+          <t xml:space="preserve">--skip-previews</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Override a safety stop (cap, open boxes, already-exists)</t>
+          <t xml:space="preserve">skip the inventory, names, ai and mcp previews</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">off</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">queue</t>
+          <t xml:space="preserve">plans</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--due</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">today|YYYY-MM-DD</t>
+          <t xml:space="preserve">--json</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">only items due on this date (today or YYYY-MM-DD)</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">all</t>
+          <t xml:space="preserve">Machine-readable JSON output</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">queue</t>
+          <t xml:space="preserve">plans</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--json</t>
+          <t xml:space="preserve">--apply</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine-readable JSON output</t>
+          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">preview</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">research</t>
+          <t xml:space="preserve">plans</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--depth</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">quick|deep</t>
+          <t xml:space="preserve">--force</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">quick answers with sources, deep starts the research-to-plan flow</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">quick</t>
+          <t xml:space="preserve">Override a safety stop (cap, open boxes, already-exists)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">research</t>
+          <t xml:space="preserve">queue</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--tool</t>
+          <t xml:space="preserve">--due</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">T</t>
+          <t xml:space="preserve">today|YYYY-MM-DD</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AI tool to use</t>
+          <t xml:space="preserve">only items due on this date (today or YYYY-MM-DD)</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">routes.default_tool (claude)</t>
+          <t xml:space="preserve">all</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">research</t>
+          <t xml:space="preserve">queue</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--dry-run</t>
+          <t xml:space="preserve">--json</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Show what would happen and change nothing</t>
+          <t xml:space="preserve">Machine-readable JSON output</t>
         </is>
       </c>
     </row>
@@ -4102,53 +4144,73 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--json</t>
+          <t xml:space="preserve">--depth</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quick|deep</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine-readable JSON output</t>
+          <t xml:space="preserve">quick answers with sources, deep starts the research-to-plan flow</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quick</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">run</t>
+          <t xml:space="preserve">research</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--dry-run</t>
+          <t xml:space="preserve">--tool</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Show what would happen and change nothing</t>
+          <t xml:space="preserve">AI tool to use</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">routes.default_tool (claude)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">run</t>
+          <t xml:space="preserve">research</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--queue</t>
+          <t xml:space="preserve">--dry-run</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Record the run as queued instead of executing it now</t>
+          <t xml:space="preserve">Show what would happen and change nothing</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">run</t>
+          <t xml:space="preserve">research</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -4170,22 +4232,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--tool</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T</t>
+          <t xml:space="preserve">--dry-run</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AI tool to use</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">routes.default_tool (claude)</t>
+          <t xml:space="preserve">Show what would happen and change nothing</t>
         </is>
       </c>
     </row>
@@ -4197,22 +4249,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--path</t>
-        </is>
-      </c>
-      <c r="C79" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P</t>
+          <t xml:space="preserve">--queue</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Working folder or project id for the run</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the working folder</t>
+          <t xml:space="preserve">Record the run as queued instead of executing it now</t>
         </is>
       </c>
     </row>
@@ -4224,22 +4266,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--machine</t>
-        </is>
-      </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">M</t>
+          <t xml:space="preserve">--json</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine to run on (a name from [machines], or any)</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">routes.default_machine (this machine)</t>
+          <t xml:space="preserve">Machine-readable JSON output</t>
         </is>
       </c>
     </row>
@@ -4251,17 +4283,22 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--write</t>
+          <t xml:space="preserve">--tool</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allow the tool to edit files (default is read-only)</t>
+          <t xml:space="preserve">AI tool to use</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">routes.permission (read-only)</t>
+          <t xml:space="preserve">routes.default_tool (claude)</t>
         </is>
       </c>
     </row>
@@ -4273,95 +4310,115 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--inbox</t>
+          <t xml:space="preserve">--path</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">run every prompt document in files/inbox/prompts not yet run</t>
+          <t xml:space="preserve">Working folder or project id for the run</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">off</t>
+          <t xml:space="preserve">the working folder</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">services</t>
+          <t xml:space="preserve">run</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--update</t>
+          <t xml:space="preserve">--machine</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">print a proposed patch for the 75/76 index files (never writes them)</t>
+          <t xml:space="preserve">Machine to run on (a name from [machines], or any)</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">off</t>
+          <t xml:space="preserve">routes.default_machine (this machine)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">sheets</t>
+          <t xml:space="preserve">run</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--json</t>
+          <t xml:space="preserve">--write</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine-readable JSON output</t>
+          <t xml:space="preserve">Allow the tool to edit files (default is read-only)</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">routes.permission (read-only)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">sheets</t>
+          <t xml:space="preserve">run</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--dry-run</t>
+          <t xml:space="preserve">--inbox</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Show what would happen and change nothing</t>
+          <t xml:space="preserve">run every prompt document in files/inbox/prompts not yet run</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">off</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">sheets</t>
+          <t xml:space="preserve">services</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--apply</t>
+          <t xml:space="preserve">--update</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
+          <t xml:space="preserve">print a proposed patch for the 75/76 index files (never writes them)</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">preview</t>
+          <t xml:space="preserve">off</t>
         </is>
       </c>
     </row>
@@ -4373,17 +4430,12 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--build</t>
+          <t xml:space="preserve">--json</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">after refresh, also run build on the set</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">off</t>
+          <t xml:space="preserve">Machine-readable JSON output</t>
         </is>
       </c>
     </row>
@@ -4395,17 +4447,12 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--check</t>
+          <t xml:space="preserve">--dry-run</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">refresh: compare the generated files with the committed ones, write nothing, exit 1 on drift</t>
-        </is>
-      </c>
-      <c r="E88" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">off</t>
+          <t xml:space="preserve">Show what would happen and change nothing</t>
         </is>
       </c>
     </row>
@@ -4417,98 +4464,88 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--out</t>
-        </is>
-      </c>
-      <c r="C89" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DIR</t>
+          <t xml:space="preserve">--apply</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">refresh: write the generated files into this folder instead of docs/</t>
+          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">docs/sheets and docs</t>
+          <t xml:space="preserve">preview</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">sheets</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--status</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">S</t>
+          <t xml:space="preserve">--build</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">only runs in this state</t>
+          <t xml:space="preserve">after refresh, also run build on the set</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">all</t>
+          <t xml:space="preserve">off</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">sheets</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">-n</t>
-        </is>
-      </c>
-      <c r="C91" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N</t>
+          <t xml:space="preserve">--check</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">number of runs to show</t>
+          <t xml:space="preserve">refresh: compare the generated files with the committed ones, write nothing, exit 1 on drift</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">off</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">sheets</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--all</t>
+          <t xml:space="preserve">--out</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DIR</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">show every run</t>
+          <t xml:space="preserve">refresh: write the generated files into this folder instead of docs/</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">off</t>
+          <t xml:space="preserve">docs/sheets and docs</t>
         </is>
       </c>
     </row>
@@ -4520,94 +4557,170 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--json</t>
+          <t xml:space="preserve">--status</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine-readable JSON output</t>
+          <t xml:space="preserve">only runs in this state</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">all</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">subsystem</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--from</t>
+          <t xml:space="preserve">-n</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">D</t>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">setup draft file to ingest (see ai-authored/templates)</t>
+          <t xml:space="preserve">number of runs to show</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">none</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">subsystem</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">--apply</t>
+          <t xml:space="preserve">--all</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
+          <t xml:space="preserve">show every run</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">preview</t>
+          <t xml:space="preserve">off</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">status</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">--json</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Machine-readable JSON output</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">subsystem</t>
         </is>
       </c>
-      <c r="B96" s="2" t="inlineStr">
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">--from</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">setup draft file to ingest (see ai-authored/templates)</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">none</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subsystem</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">--apply</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carry out the change; without it the command only previews</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subsystem</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">--replace</t>
         </is>
       </c>
-      <c r="D96" s="2" t="inlineStr">
+      <c r="D99" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">replace an existing manifest</t>
         </is>
       </c>
-      <c r="E96" s="2" t="inlineStr">
+      <c r="E99" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">off</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E96"/>
+  <autoFilter ref="A1:E99"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D453"/>
+  <dimension ref="A1:D457"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -11471,129 +11584,149 @@
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-inventory</t>
+          <t xml:space="preserve">libexec/mach-inbox</t>
         </is>
       </c>
       <c r="B372" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cleanup</t>
+          <t xml:space="preserve">drafts_json</t>
         </is>
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">bash</t>
+          <t xml:space="preserve">python</t>
         </is>
       </c>
       <c r="D372" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">shellcheck disable=SC2317 # runs through the EXIT trap</t>
+          <t xml:space="preserve">Call the official Drafts CLI and parse one JSON result.</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-inventory</t>
+          <t xml:space="preserve">libexec/mach-inbox</t>
         </is>
       </c>
       <c r="B373" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">wanted</t>
+          <t xml:space="preserve">pending</t>
         </is>
       </c>
       <c r="C373" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">bash</t>
+          <t xml:space="preserve">python</t>
         </is>
       </c>
       <c r="D373" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">wanted &lt;relative path&gt;: section filter</t>
+          <t xml:space="preserve">Yield checked documents from the tagged Drafts inbox.</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-inventory</t>
+          <t xml:space="preserve">libexec/mach-inbox</t>
         </is>
       </c>
       <c r="B374" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">protected</t>
+          <t xml:space="preserve">deliver</t>
         </is>
       </c>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">bash</t>
+          <t xml:space="preserve">python</t>
+        </is>
+      </c>
+      <c r="D374" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Save by stable Drafts ID, then archive the source only after a matching save.</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-memory</t>
+          <t xml:space="preserve">libexec/mach-inbox</t>
         </is>
       </c>
       <c r="B375" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson</t>
+          <t xml:space="preserve">main</t>
         </is>
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
+        </is>
+      </c>
+      <c r="D375" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Preview or deliver tagged drafts on the Mac.</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-memory</t>
+          <t xml:space="preserve">libexec/mach-inventory</t>
         </is>
       </c>
       <c r="B376" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson.__init__</t>
+          <t xml:space="preserve">cleanup</t>
         </is>
       </c>
       <c r="C376" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">python</t>
+          <t xml:space="preserve">bash</t>
+        </is>
+      </c>
+      <c r="D376" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">shellcheck disable=SC2317 # runs through the EXIT trap</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-memory</t>
+          <t xml:space="preserve">libexec/mach-inventory</t>
         </is>
       </c>
       <c r="B377" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson.get</t>
+          <t xml:space="preserve">wanted</t>
         </is>
       </c>
       <c r="C377" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">python</t>
+          <t xml:space="preserve">bash</t>
+        </is>
+      </c>
+      <c r="D377" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">wanted &lt;relative path&gt;: section filter</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-memory</t>
+          <t xml:space="preserve">libexec/mach-inventory</t>
         </is>
       </c>
       <c r="B378" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson.status</t>
+          <t xml:space="preserve">protected</t>
         </is>
       </c>
       <c r="C378" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">python</t>
+          <t xml:space="preserve">bash</t>
         </is>
       </c>
     </row>
@@ -11605,7 +11738,7 @@
       </c>
       <c r="B379" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson.title</t>
+          <t xml:space="preserve">Lesson</t>
         </is>
       </c>
       <c r="C379" s="2" t="inlineStr">
@@ -11622,7 +11755,7 @@
       </c>
       <c r="B380" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">lessons_root</t>
+          <t xml:space="preserve">Lesson.__init__</t>
         </is>
       </c>
       <c r="C380" s="2" t="inlineStr">
@@ -11639,7 +11772,7 @@
       </c>
       <c r="B381" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">load_cfg</t>
+          <t xml:space="preserve">Lesson.get</t>
         </is>
       </c>
       <c r="C381" s="2" t="inlineStr">
@@ -11656,7 +11789,7 @@
       </c>
       <c r="B382" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">scan</t>
+          <t xml:space="preserve">Lesson.status</t>
         </is>
       </c>
       <c r="C382" s="2" t="inlineStr">
@@ -11673,7 +11806,7 @@
       </c>
       <c r="B383" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">similar</t>
+          <t xml:space="preserve">Lesson.title</t>
         </is>
       </c>
       <c r="C383" s="2" t="inlineStr">
@@ -11690,7 +11823,7 @@
       </c>
       <c r="B384" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">scope_overlap</t>
+          <t xml:space="preserve">lessons_root</t>
         </is>
       </c>
       <c r="C384" s="2" t="inlineStr">
@@ -11707,7 +11840,7 @@
       </c>
       <c r="B385" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">contradicts</t>
+          <t xml:space="preserve">load_cfg</t>
         </is>
       </c>
       <c r="C385" s="2" t="inlineStr">
@@ -11724,17 +11857,12 @@
       </c>
       <c r="B386" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">reviews_root</t>
+          <t xml:space="preserve">scan</t>
         </is>
       </c>
       <c r="C386" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
-        </is>
-      </c>
-      <c r="D386" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Where --save writes: $MACH_REVIEWS_DIR, else [memory] reviews_dir, else &lt;lessons_dir&gt;/reviews.</t>
         </is>
       </c>
     </row>
@@ -11746,17 +11874,12 @@
       </c>
       <c r="B387" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">save_review</t>
+          <t xml:space="preserve">similar</t>
         </is>
       </c>
       <c r="C387" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
-        </is>
-      </c>
-      <c r="D387" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Write the report to reviews_dir/YYYY-MM[-N].md without clobbering; returns the path.</t>
         </is>
       </c>
     </row>
@@ -11768,7 +11891,7 @@
       </c>
       <c r="B388" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">today</t>
+          <t xml:space="preserve">scope_overlap</t>
         </is>
       </c>
       <c r="C388" s="2" t="inlineStr">
@@ -11785,7 +11908,7 @@
       </c>
       <c r="B389" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">days_between</t>
+          <t xml:space="preserve">contradicts</t>
         </is>
       </c>
       <c r="C389" s="2" t="inlineStr">
@@ -11802,12 +11925,17 @@
       </c>
       <c r="B390" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">review</t>
+          <t xml:space="preserve">reviews_root</t>
         </is>
       </c>
       <c r="C390" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
+        </is>
+      </c>
+      <c r="D390" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Where --save writes: $MACH_REVIEWS_DIR, else [memory] reviews_dir, else &lt;lessons_dir&gt;/reviews.</t>
         </is>
       </c>
     </row>
@@ -11819,12 +11947,17 @@
       </c>
       <c r="B391" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">render</t>
+          <t xml:space="preserve">save_review</t>
         </is>
       </c>
       <c r="C391" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
+        </is>
+      </c>
+      <c r="D391" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Write the report to reviews_dir/YYYY-MM[-N].md without clobbering; returns the path.</t>
         </is>
       </c>
     </row>
@@ -11836,7 +11969,7 @@
       </c>
       <c r="B392" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">apply_archives</t>
+          <t xml:space="preserve">today</t>
         </is>
       </c>
       <c r="C392" s="2" t="inlineStr">
@@ -11853,17 +11986,12 @@
       </c>
       <c r="B393" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">set_front</t>
+          <t xml:space="preserve">days_between</t>
         </is>
       </c>
       <c r="C393" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
-        </is>
-      </c>
-      <c r="D393" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Set/replace top-level keys in the frontmatter block, keeping everything else byte-for-byte.</t>
         </is>
       </c>
     </row>
@@ -11875,7 +12003,7 @@
       </c>
       <c r="B394" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">preview_collect</t>
+          <t xml:space="preserve">review</t>
         </is>
       </c>
       <c r="C394" s="2" t="inlineStr">
@@ -11892,7 +12020,7 @@
       </c>
       <c r="B395" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">preview_promote</t>
+          <t xml:space="preserve">render</t>
         </is>
       </c>
       <c r="C395" s="2" t="inlineStr">
@@ -11909,7 +12037,7 @@
       </c>
       <c r="B396" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">list_csv</t>
+          <t xml:space="preserve">apply_archives</t>
         </is>
       </c>
       <c r="C396" s="2" t="inlineStr">
@@ -11926,12 +12054,17 @@
       </c>
       <c r="B397" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">last_review</t>
+          <t xml:space="preserve">set_front</t>
         </is>
       </c>
       <c r="C397" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
+        </is>
+      </c>
+      <c r="D397" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Set/replace top-level keys in the frontmatter block, keeping everything else byte-for-byte.</t>
         </is>
       </c>
     </row>
@@ -11943,17 +12076,12 @@
       </c>
       <c r="B398" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">generate_index</t>
+          <t xml:space="preserve">preview_collect</t>
         </is>
       </c>
       <c r="C398" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
-        </is>
-      </c>
-      <c r="D398" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">INDEX.md text in the plan 09 section 4 format: header counts, then one line per proposed/active/promoted lesson per topic.</t>
         </is>
       </c>
     </row>
@@ -11965,17 +12093,12 @@
       </c>
       <c r="B399" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">init_plan</t>
+          <t xml:space="preserve">preview_promote</t>
         </is>
       </c>
       <c r="C399" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
-        </is>
-      </c>
-      <c r="D399" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Returns (dirs_to_make, files_to_make {path: text}, files_to_replace {path: text}, kept).</t>
         </is>
       </c>
     </row>
@@ -11987,7 +12110,7 @@
       </c>
       <c r="B400" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">run_init</t>
+          <t xml:space="preserve">list_csv</t>
         </is>
       </c>
       <c r="C400" s="2" t="inlineStr">
@@ -12004,7 +12127,7 @@
       </c>
       <c r="B401" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">main</t>
+          <t xml:space="preserve">last_review</t>
         </is>
       </c>
       <c r="C401" s="2" t="inlineStr">
@@ -12016,46 +12139,56 @@
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-names</t>
+          <t xml:space="preserve">libexec/mach-memory</t>
         </is>
       </c>
       <c r="B402" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">target</t>
+          <t xml:space="preserve">generate_index</t>
         </is>
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">bash</t>
+          <t xml:space="preserve">python</t>
+        </is>
+      </c>
+      <c r="D402" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INDEX.md text in the plan 09 section 4 format: header counts, then one line per proposed/active/promoted lesson per topic.</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-note</t>
+          <t xml:space="preserve">libexec/mach-memory</t>
         </is>
       </c>
       <c r="B403" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">main</t>
+          <t xml:space="preserve">init_plan</t>
         </is>
       </c>
       <c r="C403" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
+        </is>
+      </c>
+      <c r="D403" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Returns (dirs_to_make, files_to_make {path: text}, files_to_replace {path: text}, kept).</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-plans</t>
+          <t xml:space="preserve">libexec/mach-memory</t>
         </is>
       </c>
       <c r="B404" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">plans_dir</t>
+          <t xml:space="preserve">run_init</t>
         </is>
       </c>
       <c r="C404" s="2" t="inlineStr">
@@ -12067,12 +12200,12 @@
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-plans</t>
+          <t xml:space="preserve">libexec/mach-memory</t>
         </is>
       </c>
       <c r="B405" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">count_boxes</t>
+          <t xml:space="preserve">main</t>
         </is>
       </c>
       <c r="C405" s="2" t="inlineStr">
@@ -12084,29 +12217,29 @@
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-plans</t>
+          <t xml:space="preserve">libexec/mach-names</t>
         </is>
       </c>
       <c r="B406" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">status_line</t>
+          <t xml:space="preserve">target</t>
         </is>
       </c>
       <c r="C406" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">python</t>
+          <t xml:space="preserve">bash</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-plans</t>
+          <t xml:space="preserve">libexec/mach-note</t>
         </is>
       </c>
       <c r="B407" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">list_plans</t>
+          <t xml:space="preserve">main</t>
         </is>
       </c>
       <c r="C407" s="2" t="inlineStr">
@@ -12123,7 +12256,7 @@
       </c>
       <c r="B408" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">find_plan</t>
+          <t xml:space="preserve">plans_dir</t>
         </is>
       </c>
       <c r="C408" s="2" t="inlineStr">
@@ -12140,17 +12273,12 @@
       </c>
       <c r="B409" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">reference_hits</t>
+          <t xml:space="preserve">count_boxes</t>
         </is>
       </c>
       <c r="C409" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
-        </is>
-      </c>
-      <c r="D409" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Files (outside plans/archived) that mention the plan. Returns list of (path, kind, line_no, line).</t>
         </is>
       </c>
     </row>
@@ -12162,7 +12290,7 @@
       </c>
       <c r="B410" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">register_row</t>
+          <t xml:space="preserve">status_line</t>
         </is>
       </c>
       <c r="C410" s="2" t="inlineStr">
@@ -12179,7 +12307,7 @@
       </c>
       <c r="B411" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">changelog_insert</t>
+          <t xml:space="preserve">list_plans</t>
         </is>
       </c>
       <c r="C411" s="2" t="inlineStr">
@@ -12196,7 +12324,7 @@
       </c>
       <c r="B412" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cmd_list</t>
+          <t xml:space="preserve">find_plan</t>
         </is>
       </c>
       <c r="C412" s="2" t="inlineStr">
@@ -12213,12 +12341,17 @@
       </c>
       <c r="B413" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cmd_archive</t>
+          <t xml:space="preserve">reference_hits</t>
         </is>
       </c>
       <c r="C413" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
+        </is>
+      </c>
+      <c r="D413" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Files (outside plans/archived) that mention the plan. Returns list of (path, kind, line_no, line).</t>
         </is>
       </c>
     </row>
@@ -12230,7 +12363,7 @@
       </c>
       <c r="B414" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">main</t>
+          <t xml:space="preserve">register_row</t>
         </is>
       </c>
       <c r="C414" s="2" t="inlineStr">
@@ -12242,12 +12375,12 @@
     <row r="415">
       <c r="A415" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-queue</t>
+          <t xml:space="preserve">libexec/mach-plans</t>
         </is>
       </c>
       <c r="B415" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">main</t>
+          <t xml:space="preserve">changelog_insert</t>
         </is>
       </c>
       <c r="C415" s="2" t="inlineStr">
@@ -12259,12 +12392,12 @@
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-reject</t>
+          <t xml:space="preserve">libexec/mach-plans</t>
         </is>
       </c>
       <c r="B416" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">main</t>
+          <t xml:space="preserve">cmd_list</t>
         </is>
       </c>
       <c r="C416" s="2" t="inlineStr">
@@ -12276,12 +12409,12 @@
     <row r="417">
       <c r="A417" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-research</t>
+          <t xml:space="preserve">libexec/mach-plans</t>
         </is>
       </c>
       <c r="B417" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">main</t>
+          <t xml:space="preserve">cmd_archive</t>
         </is>
       </c>
       <c r="C417" s="2" t="inlineStr">
@@ -12293,12 +12426,12 @@
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-run</t>
+          <t xml:space="preserve">libexec/mach-plans</t>
         </is>
       </c>
       <c r="B418" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">report_problems</t>
+          <t xml:space="preserve">main</t>
         </is>
       </c>
       <c r="C418" s="2" t="inlineStr">
@@ -12310,12 +12443,12 @@
     <row r="419">
       <c r="A419" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-run</t>
+          <t xml:space="preserve">libexec/mach-queue</t>
         </is>
       </c>
       <c r="B419" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">flow_input</t>
+          <t xml:space="preserve">main</t>
         </is>
       </c>
       <c r="C419" s="2" t="inlineStr">
@@ -12327,12 +12460,12 @@
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-run</t>
+          <t xml:space="preserve">libexec/mach-reject</t>
         </is>
       </c>
       <c r="B420" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">run_one</t>
+          <t xml:space="preserve">main</t>
         </is>
       </c>
       <c r="C420" s="2" t="inlineStr">
@@ -12344,12 +12477,12 @@
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-run</t>
+          <t xml:space="preserve">libexec/mach-research</t>
         </is>
       </c>
       <c r="B421" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">worst</t>
+          <t xml:space="preserve">main</t>
         </is>
       </c>
       <c r="C421" s="2" t="inlineStr">
@@ -12366,7 +12499,7 @@
       </c>
       <c r="B422" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">main</t>
+          <t xml:space="preserve">report_problems</t>
         </is>
       </c>
       <c r="C422" s="2" t="inlineStr">
@@ -12378,12 +12511,12 @@
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-services</t>
+          <t xml:space="preserve">libexec/mach-run</t>
         </is>
       </c>
       <c r="B423" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">index_rows</t>
+          <t xml:space="preserve">flow_input</t>
         </is>
       </c>
       <c r="C423" s="2" t="inlineStr">
@@ -12395,34 +12528,29 @@
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-services</t>
+          <t xml:space="preserve">libexec/mach-run</t>
         </is>
       </c>
       <c r="B424" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">row_status</t>
+          <t xml:space="preserve">run_one</t>
         </is>
       </c>
       <c r="C424" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
-        </is>
-      </c>
-      <c r="D424" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Last-column status for 75, the 'Status' column (second to last) for 76.</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-services</t>
+          <t xml:space="preserve">libexec/mach-run</t>
         </is>
       </c>
       <c r="B425" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">is_active_row</t>
+          <t xml:space="preserve">worst</t>
         </is>
       </c>
       <c r="C425" s="2" t="inlineStr">
@@ -12434,22 +12562,17 @@
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-services</t>
+          <t xml:space="preserve">libexec/mach-run</t>
         </is>
       </c>
       <c r="B426" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">row_tokens</t>
+          <t xml:space="preserve">main</t>
         </is>
       </c>
       <c r="C426" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
-        </is>
-      </c>
-      <c r="D426" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Names a live item would carry: backticked words and basenames of paths in the row.</t>
         </is>
       </c>
     </row>
@@ -12461,7 +12584,7 @@
       </c>
       <c r="B427" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">live_linux</t>
+          <t xml:space="preserve">index_rows</t>
         </is>
       </c>
       <c r="C427" s="2" t="inlineStr">
@@ -12478,12 +12601,17 @@
       </c>
       <c r="B428" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">live_mac</t>
+          <t xml:space="preserve">row_status</t>
         </is>
       </c>
       <c r="C428" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
+        </is>
+      </c>
+      <c r="D428" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Last-column status for 75, the 'Status' column (second to last) for 76.</t>
         </is>
       </c>
     </row>
@@ -12495,7 +12623,7 @@
       </c>
       <c r="B429" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cron_lines</t>
+          <t xml:space="preserve">is_active_row</t>
         </is>
       </c>
       <c r="C429" s="2" t="inlineStr">
@@ -12512,12 +12640,17 @@
       </c>
       <c r="B430" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">unit_state</t>
+          <t xml:space="preserve">row_tokens</t>
         </is>
       </c>
       <c r="C430" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
+        </is>
+      </c>
+      <c r="D430" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Names a live item would carry: backticked words and basenames of paths in the row.</t>
         </is>
       </c>
     </row>
@@ -12529,7 +12662,7 @@
       </c>
       <c r="B431" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">failed_units</t>
+          <t xml:space="preserve">live_linux</t>
         </is>
       </c>
       <c r="C431" s="2" t="inlineStr">
@@ -12546,7 +12679,7 @@
       </c>
       <c r="B432" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">main</t>
+          <t xml:space="preserve">live_mac</t>
         </is>
       </c>
       <c r="C432" s="2" t="inlineStr">
@@ -12558,34 +12691,29 @@
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-sheets</t>
+          <t xml:space="preserve">libexec/mach-services</t>
         </is>
       </c>
       <c r="B433" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">report</t>
+          <t xml:space="preserve">cron_lines</t>
         </is>
       </c>
       <c r="C433" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
-        </is>
-      </c>
-      <c r="D433" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Print lint results; return the exit code (0 OK, 1 warnings, 2 failures).</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-sheets</t>
+          <t xml:space="preserve">libexec/mach-services</t>
         </is>
       </c>
       <c r="B434" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cmd_lint</t>
+          <t xml:space="preserve">unit_state</t>
         </is>
       </c>
       <c r="C434" s="2" t="inlineStr">
@@ -12597,12 +12725,12 @@
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-sheets</t>
+          <t xml:space="preserve">libexec/mach-services</t>
         </is>
       </c>
       <c r="B435" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">write_atomic</t>
+          <t xml:space="preserve">failed_units</t>
         </is>
       </c>
       <c r="C435" s="2" t="inlineStr">
@@ -12614,12 +12742,12 @@
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-sheets</t>
+          <t xml:space="preserve">libexec/mach-services</t>
         </is>
       </c>
       <c r="B436" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">do_build</t>
+          <t xml:space="preserve">main</t>
         </is>
       </c>
       <c r="C436" s="2" t="inlineStr">
@@ -12636,12 +12764,17 @@
       </c>
       <c r="B437" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cmd_new</t>
+          <t xml:space="preserve">report</t>
         </is>
       </c>
       <c r="C437" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
+        </is>
+      </c>
+      <c r="D437" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Print lint results; return the exit code (0 OK, 1 warnings, 2 failures).</t>
         </is>
       </c>
     </row>
@@ -12653,17 +12786,12 @@
       </c>
       <c r="B438" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">desired_files</t>
+          <t xml:space="preserve">cmd_lint</t>
         </is>
       </c>
       <c r="C438" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
-        </is>
-      </c>
-      <c r="D438" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">{path: text} for the refresh, plus the list of CSVs skipped because their source is missing.</t>
         </is>
       </c>
     </row>
@@ -12675,7 +12803,7 @@
       </c>
       <c r="B439" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cmd_refresh</t>
+          <t xml:space="preserve">write_atomic</t>
         </is>
       </c>
       <c r="C439" s="2" t="inlineStr">
@@ -12692,7 +12820,7 @@
       </c>
       <c r="B440" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">sh_inside</t>
+          <t xml:space="preserve">do_build</t>
         </is>
       </c>
       <c r="C440" s="2" t="inlineStr">
@@ -12709,7 +12837,7 @@
       </c>
       <c r="B441" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">main</t>
+          <t xml:space="preserve">cmd_new</t>
         </is>
       </c>
       <c r="C441" s="2" t="inlineStr">
@@ -12721,29 +12849,34 @@
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-status</t>
+          <t xml:space="preserve">libexec/mach-sheets</t>
         </is>
       </c>
       <c r="B442" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">brief</t>
+          <t xml:space="preserve">desired_files</t>
         </is>
       </c>
       <c r="C442" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
+        </is>
+      </c>
+      <c r="D442" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{path: text} for the refresh, plus the list of CSVs skipped because their source is missing.</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-status</t>
+          <t xml:space="preserve">libexec/mach-sheets</t>
         </is>
       </c>
       <c r="B443" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">main</t>
+          <t xml:space="preserve">cmd_refresh</t>
         </is>
       </c>
       <c r="C443" s="2" t="inlineStr">
@@ -12755,12 +12888,12 @@
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-subsystem</t>
+          <t xml:space="preserve">libexec/mach-sheets</t>
         </is>
       </c>
       <c r="B444" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">emit</t>
+          <t xml:space="preserve">sh_inside</t>
         </is>
       </c>
       <c r="C444" s="2" t="inlineStr">
@@ -12772,12 +12905,12 @@
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-subsystem</t>
+          <t xml:space="preserve">libexec/mach-sheets</t>
         </is>
       </c>
       <c r="B445" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">manifest</t>
+          <t xml:space="preserve">main</t>
         </is>
       </c>
       <c r="C445" s="2" t="inlineStr">
@@ -12789,12 +12922,12 @@
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-subsystem</t>
+          <t xml:space="preserve">libexec/mach-status</t>
         </is>
       </c>
       <c r="B446" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">check</t>
+          <t xml:space="preserve">brief</t>
         </is>
       </c>
       <c r="C446" s="2" t="inlineStr">
@@ -12806,12 +12939,12 @@
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">libexec/mach-subsystem</t>
+          <t xml:space="preserve">libexec/mach-status</t>
         </is>
       </c>
       <c r="B447" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">main</t>
         </is>
       </c>
       <c r="C447" s="2" t="inlineStr">
@@ -12828,7 +12961,7 @@
       </c>
       <c r="B448" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ingested</t>
+          <t xml:space="preserve">emit</t>
         </is>
       </c>
       <c r="C448" s="2" t="inlineStr">
@@ -12845,7 +12978,7 @@
       </c>
       <c r="B449" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backup_write</t>
+          <t xml:space="preserve">manifest</t>
         </is>
       </c>
       <c r="C449" s="2" t="inlineStr">
@@ -12862,7 +12995,7 @@
       </c>
       <c r="B450" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">secrets</t>
+          <t xml:space="preserve">check</t>
         </is>
       </c>
       <c r="C450" s="2" t="inlineStr">
@@ -12879,7 +13012,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">header</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
@@ -12896,7 +13029,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">curl_config</t>
+          <t xml:space="preserve">ingested</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
@@ -12913,17 +13046,85 @@
       </c>
       <c r="B453" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">backup_write</t>
+        </is>
+      </c>
+      <c r="C453" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">python</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">libexec/mach-subsystem</t>
+        </is>
+      </c>
+      <c r="B454" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">secrets</t>
+        </is>
+      </c>
+      <c r="C454" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">python</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">libexec/mach-subsystem</t>
+        </is>
+      </c>
+      <c r="B455" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">header</t>
+        </is>
+      </c>
+      <c r="C455" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">python</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">libexec/mach-subsystem</t>
+        </is>
+      </c>
+      <c r="B456" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">curl_config</t>
+        </is>
+      </c>
+      <c r="C456" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">python</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">libexec/mach-subsystem</t>
+        </is>
+      </c>
+      <c r="B457" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">send</t>
         </is>
       </c>
-      <c r="C453" s="2" t="inlineStr">
+      <c r="C457" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">python</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D453"/>
+  <autoFilter ref="A1:D457"/>
 </worksheet>
 </file>
 
@@ -13755,7 +13956,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">name of the generated Drafts action; --name overrides it</t>
+          <t xml:space="preserve">legacy; hub identity now comes from config/drafts/*.json</t>
         </is>
       </c>
     </row>
@@ -13777,7 +13978,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drafts action group to import into; empty = a stable generated id</t>
+          <t xml:space="preserve">legacy; use the adapter group_uuid instead</t>
         </is>
       </c>
     </row>

</xml_diff>